<commit_message>
G1: added data 2025
</commit_message>
<xml_diff>
--- a/2773 Monitoring.xlsx
+++ b/2773 Monitoring.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr showInkAnnotation="0" codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Public\gitrepos\decarb_monitoring\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Public\gitrepo\decarb_monitoring\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF6B899-68AB-4B2C-A431-EEDDFB2F6C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA0C1E80-C090-4045-A3FF-AEF8B82EF312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="3165" windowWidth="29040" windowHeight="17520" tabRatio="775" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="775" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kostenübersicht" sheetId="51" state="hidden" r:id="rId1"/>
@@ -35,14 +35,14 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="Reto Dettli - Persönliche Ansicht" guid="{EFCCBDBE-703D-49A8-BFD5-C70DFC4C6246}" mergeInterval="0" personalView="1" maximized="1" xWindow="182" yWindow="-1449" windowWidth="2578" windowHeight="1398" activeSheetId="1"/>
+    <customWorkbookView name="w10 Test - Persönliche Ansicht" guid="{F0C3F358-38F8-4A2B-A44F-0486E20EA4EB}" mergeInterval="0" personalView="1" xWindow="153" yWindow="43" windowWidth="1713" windowHeight="1088" activeSheetId="1"/>
+    <customWorkbookView name="Daniel Moos - Persönliche Ansicht" guid="{9D53A792-EE49-4CB1-A328-80A3B1745755}" mergeInterval="0" personalView="1" maximized="1" xWindow="1912" yWindow="-8" windowWidth="1936" windowHeight="1216" activeSheetId="1" showComments="commNone"/>
+    <customWorkbookView name="Ernst Haas - Persönliche Ansicht" guid="{E9B280C6-F6C1-4D6E-A20C-7C4266B3269C}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1916" windowHeight="923" activeSheetId="1"/>
+    <customWorkbookView name="Urs Müller - Persönliche Ansicht" guid="{684E191D-B776-4614-A9A6-09F48EE40BD1}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1916" windowHeight="978" activeSheetId="1"/>
+    <customWorkbookView name="Dmoos - Persönliche Ansicht" guid="{D178FE1B-3B10-414B-86B8-943130264B26}" mergeInterval="0" personalView="1" maximized="1" xWindow="-8" yWindow="-8" windowWidth="1936" windowHeight="1176" activeSheetId="1"/>
+    <customWorkbookView name="Andrea Binkert - Persönliche Ansicht" guid="{2A6B7D3A-520D-4798-8230-1DC17916761C}" mergeInterval="0" personalView="1" xWindow="492" windowWidth="948" windowHeight="860" activeSheetId="1"/>
     <customWorkbookView name="Basil Odermatt - Persönliche Ansicht" guid="{59C26AB4-86C6-4447-8F9F-F1FCBFE3A683}" mergeInterval="0" personalView="1" maximized="1" xWindow="2552" yWindow="-6" windowWidth="2576" windowHeight="1426" activeSheetId="1"/>
-    <customWorkbookView name="Andrea Binkert - Persönliche Ansicht" guid="{2A6B7D3A-520D-4798-8230-1DC17916761C}" mergeInterval="0" personalView="1" xWindow="492" windowWidth="948" windowHeight="860" activeSheetId="1"/>
-    <customWorkbookView name="Dmoos - Persönliche Ansicht" guid="{D178FE1B-3B10-414B-86B8-943130264B26}" mergeInterval="0" personalView="1" maximized="1" xWindow="-8" yWindow="-8" windowWidth="1936" windowHeight="1176" activeSheetId="1"/>
-    <customWorkbookView name="Urs Müller - Persönliche Ansicht" guid="{684E191D-B776-4614-A9A6-09F48EE40BD1}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1916" windowHeight="978" activeSheetId="1"/>
-    <customWorkbookView name="Ernst Haas - Persönliche Ansicht" guid="{E9B280C6-F6C1-4D6E-A20C-7C4266B3269C}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1916" windowHeight="923" activeSheetId="1"/>
-    <customWorkbookView name="Daniel Moos - Persönliche Ansicht" guid="{9D53A792-EE49-4CB1-A328-80A3B1745755}" mergeInterval="0" personalView="1" maximized="1" xWindow="1912" yWindow="-8" windowWidth="1936" windowHeight="1216" activeSheetId="1" showComments="commNone"/>
-    <customWorkbookView name="w10 Test - Persönliche Ansicht" guid="{F0C3F358-38F8-4A2B-A44F-0486E20EA4EB}" mergeInterval="0" personalView="1" xWindow="153" yWindow="43" windowWidth="1713" windowHeight="1088" activeSheetId="1"/>
-    <customWorkbookView name="Reto Dettli - Persönliche Ansicht" guid="{EFCCBDBE-703D-49A8-BFD5-C70DFC4C6246}" mergeInterval="0" personalView="1" maximized="1" xWindow="182" yWindow="-1449" windowWidth="2578" windowHeight="1398" activeSheetId="1"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1352,9 +1352,6 @@
     <t>https://disseminate.stats.swiss/rest/data/</t>
   </si>
   <si>
-    <t>CH1.GWS,DF_GWS_REG4,1.0.0/A._T._T.._T.</t>
-  </si>
-  <si>
     <t>_T,1</t>
   </si>
   <si>
@@ -1398,6 +1395,9 @@
   </si>
   <si>
     <t>CO₂-Emissionen Wärmeerzeugung kantonale Gebäude (Mietermodell) pro m2 (witterungsbereinigt)</t>
+  </si>
+  <si>
+    <t>CH1.GWS,DF_GWS_REG4,1.1.0/A._T._T.._T.</t>
   </si>
 </sst>
 </file>
@@ -2892,7 +2892,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:11" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:11" ht="104.25" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" ht="87" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>387</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>388</v>
+        <v>403</v>
       </c>
       <c r="I6" s="31"/>
       <c r="J6" s="31" t="s">
@@ -5832,7 +5832,7 @@
         <v>387</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="J12" s="25" t="s">
         <v>86</v>
@@ -5841,7 +5841,7 @@
         <v>2005</v>
       </c>
       <c r="M12" s="25" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="N12" s="25" t="s">
         <v>156</v>
@@ -5953,7 +5953,7 @@
         <v>221</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="F14" s="25" t="s">
         <v>181</v>
@@ -6123,10 +6123,10 @@
         <v>81</v>
       </c>
       <c r="C17" s="25" t="s">
+        <v>401</v>
+      </c>
+      <c r="D17" s="25" t="s">
         <v>402</v>
-      </c>
-      <c r="D17" s="25" t="s">
-        <v>403</v>
       </c>
       <c r="E17" s="25" t="s">
         <v>91</v>
@@ -6499,7 +6499,7 @@
         <v>387</v>
       </c>
       <c r="H23" s="25" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="J23" s="25" t="s">
         <v>86</v>
@@ -6509,7 +6509,7 @@
       </c>
       <c r="L23" s="25"/>
       <c r="M23" s="25" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="N23" s="25" t="s">
         <v>156</v>
@@ -6571,7 +6571,7 @@
         <v>387</v>
       </c>
       <c r="H24" s="25" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="I24" s="25"/>
       <c r="J24" s="25" t="s">
@@ -6582,7 +6582,7 @@
       </c>
       <c r="L24" s="25"/>
       <c r="M24" s="25" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="N24" s="25" t="s">
         <v>156</v>
@@ -6647,7 +6647,7 @@
         <v>387</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="I25" s="25"/>
       <c r="J25" s="25" t="s">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="L25" s="25"/>
       <c r="M25" s="25" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="N25" s="25" t="s">
         <v>156</v>
@@ -6729,7 +6729,7 @@
         <v>387</v>
       </c>
       <c r="H26" s="31" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="I26" s="31"/>
       <c r="J26" s="31" t="s">
@@ -6740,7 +6740,7 @@
       </c>
       <c r="L26" s="31"/>
       <c r="M26" s="25" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="N26" s="25" t="s">
         <v>156</v>
@@ -6811,7 +6811,7 @@
         <v>387</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="I27" s="25"/>
       <c r="J27" s="25" t="s">
@@ -6822,7 +6822,7 @@
       </c>
       <c r="L27" s="25"/>
       <c r="M27" s="25" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="N27" s="25" t="s">
         <v>156</v>
@@ -7177,7 +7177,7 @@
         <v>102</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="I32" s="25"/>
       <c r="J32" s="25" t="s">
@@ -7196,25 +7196,25 @@
         <v>156</v>
       </c>
       <c r="O32" s="25" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="P32" s="25">
         <v>16</v>
       </c>
       <c r="Q32" s="25" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="R32" s="25"/>
       <c r="S32" s="25"/>
       <c r="T32" s="25"/>
       <c r="U32" s="25" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="V32" s="25" t="s">
         <v>324</v>
       </c>
       <c r="X32" s="25" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="Y32" s="25" t="s">
         <v>159</v>
@@ -7765,15 +7765,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c16c412-41a7-483e-8458-9b4c6e041c8c">
@@ -7782,6 +7773,15 @@
     <TaxCatchAll xmlns="9ff67bf8-4dc4-49ec-8a2f-3c58a02da8ea" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7990,14 +7990,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4E4C368-1DF5-422B-BD39-8846CE2351EE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18A314DA-0F62-4E10-94F7-DBFCC9F3B707}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -8010,6 +8002,14 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4E4C368-1DF5-422B-BD39-8846CE2351EE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>